<commit_message>
Additional bindings par cas d'usage sur Condition.code
Remplace le ValueSet agrégé FRCoreValueSetConditionCode par 4 ValueSets
par cas d'usage (défaut, allergie, médecine de ville, maladie rare),
documentés via le mécanisme FHIR des additional bindings (purpose
extensible) sur Condition.code, à l'image de condition-eu-core.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> e4939ed823b226ca51854e897167cf4a3cec2d42
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-14T12:24:46+00:00</t>
+    <t>2026-09-14T12:47:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -785,7 +785,7 @@
     <t>extensible</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-condition-code|2.2.0</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-condition-code-defaut|2.2.0</t>
   </si>
   <si>
     <t>Event.code</t>

</xml_diff>

<commit_message>
fix: retire le binding allergie/hypersensibilité de Condition.code, redirige vers AllergyIntolerance
Les réactions allergiques, hypersensibilités non allergiques, intolérances
et idiosyncrasies doivent être portées par AllergyIntolerance, pas par
Condition. Supprime l'additional binding CIM-11 Chapitre 04 devenu
incorrect côté Condition et le ValueSet fr-core-vs-condition-code-allergie
associé (désormais géré côté fr-core-allergy-intolerance). Documente le
choix de ressource dans code ^definition.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> e69a553d2339c239acb6e8d534e26d5a28c3eb9b
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-16T08:14:25+00:00</t>
+    <t>2026-09-16T15:45:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -774,7 +774,7 @@
   </si>
   <si>
     <t>CIM-10 pour les pathologies et réactions à une vaccination : Si le problème observé n'est pas trouvé dans la terminologie CIM-10, utiliser le code='R69' display='Causes inconnues et non précisées de morbidité' system='https://smt.esante.gouv.fr/terminologie-cim-10' et décrire le problème sous forme de texte libre.
-Réaction allergique : CIM-11 / Chapitre 04 Maladies du système immunitaire / Bloc Affections allergiques ou d'hyper-sensibilité.
+Allergie, hypersensibilité non allergique, intolérance ou idiosyncrasie : ne pas utiliser Condition — utiliser la ressource AllergyIntolerance (FRCoreAllergyIntoleranceProfile).
 Maladie rare : ORPHAcode (Orphanet) - system='https://www.orpha.net'.
 Si pas de problème ou pas d'information : https://smt.esante.gouv.fr/fhir/ValueSet/jdv-absent-or-unknown-problem-cisis</t>
   </si>

</xml_diff>

<commit_message>
Fix exemple Condition : stage.summary doit utiliser la slice clinicalStatus
stage.summary était renseigné sans stage.type, donc ne matchait pas le
discriminator pattern de la slice clinicalStatus sur Condition.stage.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 31e6303e0cbd91767eecdaa01e55d3bf088841bc
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
+++ b/nr-doc-core-condition/ig/StructureDefinition-fr-core-condition.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-17T13:23:37+00:00</t>
+    <t>2026-10-13T12:11:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -718,7 +718,7 @@
     <t>The categorization is often highly contextual and may appear poorly differentiated or not very useful in other contexts.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260716085853</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-code-probleme-cisis|20260916095457</t>
   </si>
   <si>
     <t>&lt; 404684003 |Clinical finding|</t>
@@ -1285,7 +1285,7 @@
     <t>Statut clinique du patient</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260716085852</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-health-status-code-cisis|20260916095455</t>
   </si>
   <si>
     <t>Condition.stage:clinicalStatus.assessment</t>

</xml_diff>